<commit_message>
Updated predictor prep process
</commit_message>
<xml_diff>
--- a/tools/model_specs.xlsx
+++ b/tools/model_specs.xlsx
@@ -1,94 +1,101 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <workbookPr date1904="false"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20392"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\LULCC_CH\Tools\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADC57BA7-C0CE-442D-90A3-F49DE4F7860A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="0"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet 1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
-  <si>
-    <t xml:space="preserve">Data_period_name</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gen_model_tag</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Detail_model_tag</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Model_type</t>
-  </si>
-  <si>
-    <t xml:space="preserve">model_scale</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Feature_selection_employed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">balance_adjustment</t>
-  </si>
-  <si>
-    <t xml:space="preserve">subset_nhood</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nhood_extent</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Modelling_completed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Period_1985_1997</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rf_regionalized_filtered</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Period_1985_1997.rf_regionalized_filtered.downsampled</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">regionalized</t>
-  </si>
-  <si>
-    <t xml:space="preserve">downsampled</t>
-  </si>
-  <si>
-    <t xml:space="preserve">N</t>
-  </si>
-  <si>
-    <t xml:space="preserve">na</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Period_1997_2009</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Period_1997_2009.rf_regionalized_filtered.downsampled</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Period_2009_2018</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Period_2009_2018.rf_regionalized_filtered.downsampled</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Y</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="23">
+  <si>
+    <t>Data_period_name</t>
+  </si>
+  <si>
+    <t>Gen_model_tag</t>
+  </si>
+  <si>
+    <t>Detail_model_tag</t>
+  </si>
+  <si>
+    <t>Model_type</t>
+  </si>
+  <si>
+    <t>model_scale</t>
+  </si>
+  <si>
+    <t>Feature_selection_employed</t>
+  </si>
+  <si>
+    <t>balance_adjustment</t>
+  </si>
+  <si>
+    <t>subset_nhood</t>
+  </si>
+  <si>
+    <t>Nhood_extent</t>
+  </si>
+  <si>
+    <t>Modelling_completed</t>
+  </si>
+  <si>
+    <t>rf_regionalized_filtered</t>
+  </si>
+  <si>
+    <t>Period_1985_1997.rf_regionalized_filtered.downsampled</t>
+  </si>
+  <si>
+    <t>rf</t>
+  </si>
+  <si>
+    <t>regionalized</t>
+  </si>
+  <si>
+    <t>downsampled</t>
+  </si>
+  <si>
+    <t>N</t>
+  </si>
+  <si>
+    <t>na</t>
+  </si>
+  <si>
+    <t>Period_1997_2009.rf_regionalized_filtered.downsampled</t>
+  </si>
+  <si>
+    <t>Period_2009_2018.rf_regionalized_filtered.downsampled</t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>1985_1997</t>
+  </si>
+  <si>
+    <t>1997_2009</t>
+  </si>
+  <si>
+    <t>2009_2018</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -124,6 +131,15 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -405,11 +421,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:J4"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="35.140625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -441,104 +460,104 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" t="s">
         <v>10</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>11</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>12</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>13</v>
-      </c>
-      <c r="E2" t="s">
-        <v>14</v>
       </c>
       <c r="F2" t="b">
         <v>1</v>
       </c>
       <c r="G2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H2" t="s">
         <v>15</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>16</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" t="s">
         <v>17</v>
       </c>
-      <c r="J2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="s">
-        <v>18</v>
-      </c>
-      <c r="B3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" t="s">
-        <v>19</v>
-      </c>
       <c r="D3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" t="s">
         <v>13</v>
-      </c>
-      <c r="E3" t="s">
-        <v>14</v>
       </c>
       <c r="F3" t="b">
         <v>1</v>
       </c>
       <c r="G3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H3" t="s">
         <v>15</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>16</v>
       </c>
-      <c r="I3" t="s">
-        <v>17</v>
-      </c>
       <c r="J3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C4" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" t="s">
         <v>13</v>
-      </c>
-      <c r="E4" t="s">
-        <v>14</v>
       </c>
       <c r="F4" t="b">
         <v>1</v>
       </c>
       <c r="G4" t="s">
+        <v>14</v>
+      </c>
+      <c r="H4" t="s">
         <v>15</v>
       </c>
-      <c r="H4" t="s">
+      <c r="I4" t="s">
         <v>16</v>
       </c>
-      <c r="I4" t="s">
-        <v>17</v>
-      </c>
       <c r="J4" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
config + initial testing infra
</commit_message>
<xml_diff>
--- a/tools/model_specs.xlsx
+++ b/tools/model_specs.xlsx
@@ -1,54 +1,40 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20394"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10119"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\LULCC_CH\Tools\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jhartman/github-repos/evoland-with-baggage/tools/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7130621-85EF-4B5F-9119-83C95A0F98FD}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D2A9A69-298B-FD4C-95D9-0AFF1539A2A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="13130" windowHeight="6110" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="20">
   <si>
-    <t>Data_period_name</t>
-  </si>
-  <si>
-    <t>Gen_model_tag</t>
-  </si>
-  <si>
-    <t>Detail_model_tag</t>
-  </si>
-  <si>
-    <t>Model_type</t>
-  </si>
-  <si>
-    <t>Model_scale</t>
-  </si>
-  <si>
-    <t>Feature_selection_employed</t>
-  </si>
-  <si>
-    <t>Balance_adjustment</t>
-  </si>
-  <si>
-    <t>Nhood_extent</t>
-  </si>
-  <si>
-    <t>Modelling_completed</t>
-  </si>
-  <si>
     <t>1985_1997</t>
   </si>
   <si>
@@ -80,6 +66,33 @@
   </si>
   <si>
     <t>Y</t>
+  </si>
+  <si>
+    <t>data_period_name</t>
+  </si>
+  <si>
+    <t>gen_model_tag</t>
+  </si>
+  <si>
+    <t>detail_model_tag</t>
+  </si>
+  <si>
+    <t>model_type</t>
+  </si>
+  <si>
+    <t>model_scale</t>
+  </si>
+  <si>
+    <t>feature_selection_employed</t>
+  </si>
+  <si>
+    <t>balance_adjustment</t>
+  </si>
+  <si>
+    <t>nhood_extent</t>
+  </si>
+  <si>
+    <t>modelling_completed</t>
   </si>
 </sst>
 </file>
@@ -414,122 +427,122 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I4"/>
-  <sheetFormatPr defaultColWidth="10.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E1" t="s">
+        <v>15</v>
+      </c>
+      <c r="F1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1" t="s">
+        <v>17</v>
+      </c>
+      <c r="H1" t="s">
+        <v>18</v>
+      </c>
+      <c r="I1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F2" t="b">
+        <v>1</v>
+      </c>
+      <c r="G2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="I2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="B3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="D3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F3" t="b">
+        <v>1</v>
+      </c>
+      <c r="G3" t="b">
+        <v>1</v>
+      </c>
+      <c r="H3" t="s">
+        <v>5</v>
+      </c>
+      <c r="I3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+      <c r="B4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C4" t="s">
         <v>9</v>
       </c>
-      <c r="B2" t="s">
+      <c r="D4" t="s">
+        <v>3</v>
+      </c>
+      <c r="E4" t="s">
+        <v>4</v>
+      </c>
+      <c r="F4" t="b">
+        <v>1</v>
+      </c>
+      <c r="G4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H4" t="s">
+        <v>5</v>
+      </c>
+      <c r="I4" t="s">
         <v>10</v>
-      </c>
-      <c r="C2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E2" t="s">
-        <v>13</v>
-      </c>
-      <c r="F2" t="b">
-        <v>1</v>
-      </c>
-      <c r="G2" t="b">
-        <v>1</v>
-      </c>
-      <c r="H2" t="s">
-        <v>14</v>
-      </c>
-      <c r="I2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D3" t="s">
-        <v>12</v>
-      </c>
-      <c r="E3" t="s">
-        <v>13</v>
-      </c>
-      <c r="F3" t="b">
-        <v>1</v>
-      </c>
-      <c r="G3" t="b">
-        <v>1</v>
-      </c>
-      <c r="H3" t="s">
-        <v>14</v>
-      </c>
-      <c r="I3" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B4" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" t="s">
-        <v>18</v>
-      </c>
-      <c r="D4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E4" t="s">
-        <v>13</v>
-      </c>
-      <c r="F4" t="b">
-        <v>1</v>
-      </c>
-      <c r="G4" t="b">
-        <v>1</v>
-      </c>
-      <c r="H4" t="s">
-        <v>14</v>
-      </c>
-      <c r="I4" t="s">
-        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
7 transition modelling (#17)
* #7 first pass

* #7 deep into the belly of the beast

* #7 seems that this model lookup table is discarded in _finalization

* #7 have no found any actual usage for the extracted models

* #7 cleanup, documentation

* #7 successful transition_modelling runthrough

* importing Model_evaluation.R from ICoLCM

* line breaks for legibility

* legibility, linter complaints, dead code

* modelstatscomparison: namespaces, linelengths

* #7 final step for prediction modelling
</commit_message>
<xml_diff>
--- a/tools/model_specs.xlsx
+++ b/tools/model_specs.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10119"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jhartman/github-repos/evoland-with-baggage/tools/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D2A9A69-298B-FD4C-95D9-0AFF1539A2A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CC7CD4F-4042-C645-9C3E-98E0009AA392}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -65,9 +65,6 @@
     <t>Period_2009_2018.rf_regionalized_filtered.downsampled</t>
   </si>
   <si>
-    <t>Y</t>
-  </si>
-  <si>
     <t>data_period_name</t>
   </si>
   <si>
@@ -93,6 +90,9 @@
   </si>
   <si>
     <t>modelling_completed</t>
+  </si>
+  <si>
+    <t>N</t>
   </si>
 </sst>
 </file>
@@ -431,31 +431,31 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" t="s">
         <v>11</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>12</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>13</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>14</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>15</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>16</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>17</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>18</v>
-      </c>
-      <c r="I1" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.2">
@@ -484,7 +484,7 @@
         <v>5</v>
       </c>
       <c r="I2" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
@@ -513,7 +513,7 @@
         <v>5</v>
       </c>
       <c r="I3" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
@@ -542,7 +542,7 @@
         <v>5</v>
       </c>
       <c r="I4" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>